<commit_message>
Mejora de la vista del login. el panel admin, y de la vista del registro. Creacion un Dashboard con barra y dona.
</commit_message>
<xml_diff>
--- a/reporte_calibraciones.xlsx
+++ b/reporte_calibraciones.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -942,6 +942,33 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Tecnico</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>agregado desde panel del tecnico</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2027-05-05</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>